<commit_message>
Add FortuneSheet-aligned DataGrid M3: styles, freeze, copy/fill
Parse styles.xml into CellStyle (fill/font/align/numFmt), honour sheet
freeze panes with fixed bands, and wire Ctrl+C/V TSV plus fill-handle
copy-fill — all grounded in the FortuneSheet feature checklist.

Co-authored-by: Tero <terotests@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fixtures/sales.xlsx
+++ b/fixtures/sales.xlsx
@@ -39,25 +39,50 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
     <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -72,21 +97,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -97,10 +122,10 @@
       <c r="B3">
         <v>12</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>4.5</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <f>B3*C3</f>
         <v>54</v>
       </c>
@@ -112,10 +137,10 @@
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>19.9</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <f>B4*C4</f>
         <v>59.7</v>
       </c>
@@ -127,10 +152,10 @@
       <c r="B5">
         <v>100</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="3">
         <v>0.25</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <f>B5*C5</f>
         <v>25</v>
       </c>
@@ -141,7 +166,7 @@
           <t>Grand total</t>
         </is>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <f>SUM(D3:D5)</f>
         <v>138.7</v>
       </c>

</xml_diff>